<commit_message>
Updated ABARES forecast for 2025-26
</commit_message>
<xml_diff>
--- a/data/Chickpea_production_1989_2025.xlsx
+++ b/data/Chickpea_production_1989_2025.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://griffitheduau-my.sharepoint.com/personal/i_bar_griffith_edu_au/Documents/Research/Crop_production/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="90" documentId="11_F4A336343DFE732C531AFCADFBA2C6AC91DFBD02" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{241A9B3D-EF55-49D4-A8E5-4ECD9F8604F8}"/>
+  <xr:revisionPtr revIDLastSave="136" documentId="11_F4A336343DFE732C531AFCADFBA2C6AC91DFBD02" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A50578E-B7DC-4786-B31B-B4B93744F88C}"/>
   <bookViews>
-    <workbookView xWindow="63465" yWindow="4215" windowWidth="17280" windowHeight="8880" firstSheet="3" activeTab="5" xr2:uid="{AF1EB0A9-8152-4A6D-A7DF-04592E58EBBE}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" firstSheet="4" activeTab="6" xr2:uid="{AF1EB0A9-8152-4A6D-A7DF-04592E58EBBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Chickpea_prod_updated" sheetId="6" r:id="rId1"/>
     <sheet name="Chickpea_prices_qrtr" sheetId="7" r:id="rId2"/>
-    <sheet name="Chickpea_prices_yr" sheetId="2" r:id="rId3"/>
-    <sheet name="Chickpea_prod_yearly" sheetId="3" r:id="rId4"/>
-    <sheet name="Chickpea_area_yearly" sheetId="4" r:id="rId5"/>
-    <sheet name="Chickpea_yield_yearly" sheetId="5" r:id="rId6"/>
+    <sheet name="Chickpea_prices_yr" sheetId="8" r:id="rId3"/>
+    <sheet name="Chickpea_prices_yr_old" sheetId="2" r:id="rId4"/>
+    <sheet name="Chickpea_prod_yearly" sheetId="3" r:id="rId5"/>
+    <sheet name="Chickpea_area_yearly" sheetId="4" r:id="rId6"/>
+    <sheet name="Chickpea_yield_yearly" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="61">
   <si>
     <t>State</t>
   </si>
@@ -210,6 +211,21 @@
   <si>
     <t>2024-2025</t>
   </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>2025–26 f</t>
+  </si>
+  <si>
+    <t>Price_domestic</t>
+  </si>
+  <si>
+    <t>Price_export</t>
+  </si>
+  <si>
+    <t>1988–89</t>
+  </si>
 </sst>
 </file>
 
@@ -219,7 +235,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="[$$-C09]#,##0.00;[Red]&quot;-&quot;[$$-C09]#,##0.00"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -444,8 +460,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri Light"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -637,8 +660,14 @@
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -782,6 +811,17 @@
       <bottom style="thin">
         <color theme="4" tint="0.39997558519241921"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1016,7 +1056,7 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1028,6 +1068,10 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="3" fontId="32" fillId="35" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="195">
     <cellStyle name="20% - Accent1" xfId="24" builtinId="30" customBuiltin="1"/>
@@ -1226,43 +1270,7 @@
     <cellStyle name="Total" xfId="22" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="19" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="31">
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
+  <dxfs count="108">
     <dxf>
       <font>
         <b val="0"/>
@@ -1274,41 +1282,35 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <sz val="9.5"/>
+        <color indexed="8"/>
+        <name val="Calibri Light"/>
+        <family val="1"/>
+        <scheme val="major"/>
       </font>
       <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
         <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
+          <color theme="0"/>
         </top>
         <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
+          <color theme="0"/>
         </bottom>
         <vertical/>
         <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1322,40 +1324,279 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
+        <sz val="9.5"/>
+        <color indexed="8"/>
+        <name val="Calibri Light"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="###\ ##0.0;\–###\ ##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFFFFFFF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFFFFFFF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFFFFFFF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFFFFFFF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9.5"/>
+        <color indexed="8"/>
+        <name val="Calibri Light"/>
+        <family val="1"/>
+        <scheme val="major"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
+          <fgColor indexed="64"/>
+          <bgColor indexed="9"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="#,##0;\–#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="0.0;\–0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="#,##0;\–#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="#,##0;\–#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="#,##0;\–#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="0.0;\–0.0"/>
     </dxf>
     <dxf>
       <font>
@@ -1444,97 +1685,57 @@
     <dxf>
       <border outline="0">
         <bottom style="thin">
-          <color theme="0"/>
+          <color rgb="FFFFFFFF"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9.5"/>
-        <color indexed="8"/>
-        <name val="Calibri Light"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right style="thin">
-          <color theme="0"/>
-        </right>
-        <top style="thin">
-          <color theme="0"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9.5"/>
-        <color indexed="8"/>
-        <name val="Calibri Light"/>
-        <family val="1"/>
-        <scheme val="major"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right style="thin">
-          <color theme="0"/>
-        </right>
-        <top/>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
     </dxf>
     <dxf>
       <font>
@@ -1549,14 +1750,14 @@
         <vertAlign val="baseline"/>
         <sz val="8"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
+        <name val="Calibri Light"/>
+        <family val="1"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="166" formatCode="###\ ##0.0;\–###\ ##0"/>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
+          <fgColor indexed="64"/>
           <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
@@ -1589,29 +1790,185 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="9.5"/>
-        <color indexed="8"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
         <name val="Calibri Light"/>
         <family val="1"/>
-        <scheme val="major"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFFFFFFF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFFFFFFF"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFFFFFFF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0;\-0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor indexed="9"/>
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right style="thin">
-          <color theme="0"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1627,9 +1984,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7D302CF3-8E88-4576-B3C1-E3516F47C220}" name="Table17" displayName="Table17" ref="A1:AL11" totalsRowShown="0" headerRowDxfId="30">
-  <autoFilter ref="A1:AL11" xr:uid="{E8A78859-0DB2-45A8-8B78-0FB949CC6D01}"/>
-  <tableColumns count="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7D302CF3-8E88-4576-B3C1-E3516F47C220}" name="Table17" displayName="Table17" ref="A1:AM11" totalsRowShown="0" headerRowDxfId="8">
+  <autoFilter ref="A1:AM11" xr:uid="{E8A78859-0DB2-45A8-8B78-0FB949CC6D01}"/>
+  <tableColumns count="39">
     <tableColumn id="1" xr3:uid="{6200B5BD-D43C-4FE6-B21D-5755B9F9210E}" name="State"/>
     <tableColumn id="2" xr3:uid="{B0DB6907-DDAD-4C81-9D2A-85C8D6C71AC6}" name="Measure"/>
     <tableColumn id="3" xr3:uid="{B53197FC-D93C-432B-B0E1-4EC1444EC7C6}" name="1989–90"/>
@@ -1665,80 +2022,98 @@
     <tableColumn id="33" xr3:uid="{3AC3CD7C-2737-4D3F-9D8D-2E6539ADB566}" name="2019–20"/>
     <tableColumn id="34" xr3:uid="{ACB3D021-B3E6-402F-80EA-21148172803A}" name="2020–21"/>
     <tableColumn id="35" xr3:uid="{FBEB0465-45EB-4FA7-A285-ABB776B487F5}" name="2021–22"/>
-    <tableColumn id="36" xr3:uid="{56290233-00EB-47A4-8350-7CFF2A31E617}" name="2022–23 s" dataDxfId="29"/>
+    <tableColumn id="36" xr3:uid="{56290233-00EB-47A4-8350-7CFF2A31E617}" name="2022–23 s" dataDxfId="7"/>
     <tableColumn id="37" xr3:uid="{2E7206F2-22F3-4807-BAA7-3AC71C333DEB}" name="2023–24 s"/>
     <tableColumn id="38" xr3:uid="{2578F50D-7F04-419B-8BC1-A2E80B9DCDD4}" name="2024–25 s"/>
+    <tableColumn id="39" xr3:uid="{4693FB47-9C18-43BE-9EAE-650E712532B0}" name="2025–26 f"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B6FB41E5-0B95-4039-98E4-98EE70E05107}" name="Table22" displayName="Table22" ref="A1:C121" totalsRowShown="0" tableBorderDxfId="28">
-  <autoFilter ref="A1:C121" xr:uid="{5224B8B4-49D9-4E03-8639-2E4604D735B3}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{5AFE1D09-28E0-4A8A-BD86-A778BDA959A6}" name="Year" dataDxfId="27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B6FB41E5-0B95-4039-98E4-98EE70E05107}" name="Table22" displayName="Table22" ref="A1:D124" totalsRowShown="0" tableBorderDxfId="2">
+  <autoFilter ref="A1:D124" xr:uid="{5224B8B4-49D9-4E03-8639-2E4604D735B3}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{5AFE1D09-28E0-4A8A-BD86-A778BDA959A6}" name="Year" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{94A7FA29-9DF9-464A-AE1C-9C7DFE4240AD}" name="Quarter"/>
-    <tableColumn id="2" xr3:uid="{A5A576D0-761B-4FDB-BE9B-A91E97D5A415}" name="Price" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{A5A576D0-761B-4FDB-BE9B-A91E97D5A415}" name="Price_domestic" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{560E2353-38B9-426E-B598-DB0F2724E37F}" name="Price_export"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{23C009A5-0511-400B-BE4C-C924101E19CD}" name="Table2" displayName="Table2" ref="A1:E37" totalsRowShown="0" tableBorderDxfId="25">
-  <autoFilter ref="A1:E37" xr:uid="{5224B8B4-49D9-4E03-8639-2E4604D735B3}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{CFF3BD70-0A12-48F8-8352-A5AEC2BD5387}" name="Period" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{A1EAACBC-FBC2-4B57-99F7-B977ED029A3E}" name="Price" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{1961752F-0F04-4162-8ECF-67DCB669F5FB}" name="Export"/>
-    <tableColumn id="4" xr3:uid="{CBF5AC75-2AC5-4747-AEFE-09493100FC68}" name="Area"/>
-    <tableColumn id="5" xr3:uid="{CE2F7C19-8D5F-45CD-8B00-233D81217571}" name="Production"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C116F515-FB52-45A5-B01E-29BF10801B58}" name="Table28" displayName="Table28" ref="A1:F40" totalsRowShown="0" tableBorderDxfId="61">
+  <autoFilter ref="A1:F40" xr:uid="{5224B8B4-49D9-4E03-8639-2E4604D735B3}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{F39B0A13-63A0-44D5-AA45-AE93F786A917}" name="Period" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{F4275F08-C195-40D3-B22B-BAE1B812ED17}" name="Price" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{881C1FD5-49D7-4015-ABA2-585782F37CC2}" name="Export"/>
+    <tableColumn id="4" xr3:uid="{E41B0F62-2A04-4525-9831-9386A49175D1}" name="Area"/>
+    <tableColumn id="5" xr3:uid="{D91D2F7D-520F-49B6-B68F-70D79790A9FC}" name="Production"/>
+    <tableColumn id="6" xr3:uid="{AE8ACA2D-BCC0-4C48-933E-2BA5383E14FC}" name="Value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6B95E510-1A8A-439E-BC61-88A4BD1030FB}" name="Table3" displayName="Table3" ref="A1:F37" totalsRowShown="0" headerRowDxfId="22">
-  <autoFilter ref="A1:F37" xr:uid="{6B95E510-1A8A-439E-BC61-88A4BD1030FB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{23C009A5-0511-400B-BE4C-C924101E19CD}" name="Table2" displayName="Table2" ref="A1:F39" totalsRowShown="0" tableBorderDxfId="80">
+  <autoFilter ref="A1:F39" xr:uid="{5224B8B4-49D9-4E03-8639-2E4604D735B3}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C042FA25-48C7-4187-AA4E-C00C0E1F087B}" name="Year" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{B02DB98D-CEEA-4199-8732-BB7027040B24}" name="New South Wales" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{05BFBAAF-E20C-4B40-9B69-B281EDF7F548}" name="Victoria" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{08CE00D7-E0CA-4A99-A532-B90C0BF0C1AD}" name="Queensland" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{85259DDA-A73B-45C4-9B0C-0B01A112B469}" name="South Australia" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{EF4CF4AF-AF79-49D4-B204-07B40A410C03}" name="Western Australia" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{CFF3BD70-0A12-48F8-8352-A5AEC2BD5387}" name="Period" dataDxfId="79"/>
+    <tableColumn id="2" xr3:uid="{A1EAACBC-FBC2-4B57-99F7-B977ED029A3E}" name="Price" dataDxfId="78"/>
+    <tableColumn id="3" xr3:uid="{1961752F-0F04-4162-8ECF-67DCB669F5FB}" name="Export"/>
+    <tableColumn id="4" xr3:uid="{CBF5AC75-2AC5-4747-AEFE-09493100FC68}" name="Area"/>
+    <tableColumn id="5" xr3:uid="{CE2F7C19-8D5F-45CD-8B00-233D81217571}" name="Production"/>
+    <tableColumn id="6" xr3:uid="{035E9FEE-10AC-48D8-9410-AB7B4A4E2BF7}" name="Value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{578CD9E2-7B2A-4D03-87FA-645F79142B74}" name="Table5" displayName="Table5" ref="A1:F37" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13">
-  <autoFilter ref="A1:F37" xr:uid="{578CD9E2-7B2A-4D03-87FA-645F79142B74}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6B95E510-1A8A-439E-BC61-88A4BD1030FB}" name="Table3" displayName="Table3" ref="A1:F37" totalsRowShown="0" headerRowDxfId="107">
+  <autoFilter ref="A1:F37" xr:uid="{6B95E510-1A8A-439E-BC61-88A4BD1030FB}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{11200E24-A2C9-4D3B-AD13-ADA099D43133}" name="Year" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{944953C7-1820-4EEB-B2B3-8F179986ECC9}" name="New South Wales" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{0A4B789D-B62E-4A30-A27B-C18F7732066C}" name="Victoria" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{BE01B1B3-5080-468C-A883-42FE45B6F193}" name="Queensland" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{53969DA5-57E3-4CE5-B68D-990DFC0B34E9}" name="South Australia" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{E9E70CB9-31D9-4B47-90BB-9DD82B5F5230}" name="Western Australia" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{C042FA25-48C7-4187-AA4E-C00C0E1F087B}" name="Year" dataDxfId="106"/>
+    <tableColumn id="2" xr3:uid="{B02DB98D-CEEA-4199-8732-BB7027040B24}" name="New South Wales" dataDxfId="105"/>
+    <tableColumn id="3" xr3:uid="{05BFBAAF-E20C-4B40-9B69-B281EDF7F548}" name="Victoria" dataDxfId="104"/>
+    <tableColumn id="4" xr3:uid="{08CE00D7-E0CA-4A99-A532-B90C0BF0C1AD}" name="Queensland" dataDxfId="103"/>
+    <tableColumn id="5" xr3:uid="{85259DDA-A73B-45C4-9B0C-0B01A112B469}" name="South Australia" dataDxfId="102"/>
+    <tableColumn id="6" xr3:uid="{EF4CF4AF-AF79-49D4-B204-07B40A410C03}" name="Western Australia" dataDxfId="101"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0ABB3E23-7A29-41EC-8A13-0A1FFD23E015}" name="Table35" displayName="Table35" ref="A1:F38" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{578CD9E2-7B2A-4D03-87FA-645F79142B74}" name="Table5" displayName="Table5" ref="A1:F37" totalsRowShown="0" headerRowDxfId="100" headerRowBorderDxfId="99" tableBorderDxfId="98">
+  <autoFilter ref="A1:F37" xr:uid="{578CD9E2-7B2A-4D03-87FA-645F79142B74}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{11200E24-A2C9-4D3B-AD13-ADA099D43133}" name="Year" dataDxfId="97"/>
+    <tableColumn id="2" xr3:uid="{944953C7-1820-4EEB-B2B3-8F179986ECC9}" name="New South Wales" dataDxfId="96"/>
+    <tableColumn id="3" xr3:uid="{0A4B789D-B62E-4A30-A27B-C18F7732066C}" name="Victoria" dataDxfId="95"/>
+    <tableColumn id="4" xr3:uid="{BE01B1B3-5080-468C-A883-42FE45B6F193}" name="Queensland" dataDxfId="94"/>
+    <tableColumn id="5" xr3:uid="{53969DA5-57E3-4CE5-B68D-990DFC0B34E9}" name="South Australia" dataDxfId="93"/>
+    <tableColumn id="6" xr3:uid="{E9E70CB9-31D9-4B47-90BB-9DD82B5F5230}" name="Western Australia" dataDxfId="92"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0ABB3E23-7A29-41EC-8A13-0A1FFD23E015}" name="Table35" displayName="Table35" ref="A1:F38" totalsRowShown="0" headerRowDxfId="91">
   <autoFilter ref="A1:F38" xr:uid="{0ABB3E23-7A29-41EC-8A13-0A1FFD23E015}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{8F263118-8E0D-4C09-9AFC-D01491D6E376}" name="Year" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{CA0488E5-A57C-47C3-A22B-509ED397FE43}" name="New South Wales" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{68D15EAE-C905-4751-81CD-60E497FDBCF5}" name="Victoria" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{0E854138-7B8A-43E6-A83D-BEFBC32927E1}" name="Queensland" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{F5E8BF13-AEF4-4260-8C7E-F6D10A57D26B}" name="South Australia" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{1453E456-0201-4E58-9A62-7C17F7993DD8}" name="Western Australia" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{8F263118-8E0D-4C09-9AFC-D01491D6E376}" name="Year" dataDxfId="90"/>
+    <tableColumn id="2" xr3:uid="{CA0488E5-A57C-47C3-A22B-509ED397FE43}" name="New South Wales" dataDxfId="89"/>
+    <tableColumn id="3" xr3:uid="{68D15EAE-C905-4751-81CD-60E497FDBCF5}" name="Victoria" dataDxfId="88"/>
+    <tableColumn id="4" xr3:uid="{0E854138-7B8A-43E6-A83D-BEFBC32927E1}" name="Queensland" dataDxfId="87"/>
+    <tableColumn id="5" xr3:uid="{F5E8BF13-AEF4-4260-8C7E-F6D10A57D26B}" name="South Australia" dataDxfId="86"/>
+    <tableColumn id="6" xr3:uid="{1453E456-0201-4E58-9A62-7C17F7993DD8}" name="Western Australia" dataDxfId="85"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2041,7 +2416,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4550E558-D337-45FB-AAE5-044546BF41F8}">
-  <dimension ref="A1:AL11"/>
+  <dimension ref="A1:AM11"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
@@ -2057,7 +2432,7 @@
     <col min="18" max="18" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38">
+    <row r="1" spans="1:39">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2172,8 +2547,11 @@
       <c r="AL1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="2" spans="1:38">
+      <c r="AM1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:39">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2288,8 +2666,11 @@
       <c r="AL2">
         <v>580</v>
       </c>
-    </row>
-    <row r="3" spans="1:38">
+      <c r="AM2">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="3" spans="1:39">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2404,8 +2785,11 @@
       <c r="AL3">
         <v>1280</v>
       </c>
-    </row>
-    <row r="4" spans="1:38">
+      <c r="AM3">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="4" spans="1:39">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -2520,8 +2904,11 @@
       <c r="AL4">
         <v>420</v>
       </c>
-    </row>
-    <row r="5" spans="1:38">
+      <c r="AM4">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="5" spans="1:39">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -2636,8 +3023,11 @@
       <c r="AL5">
         <v>950</v>
       </c>
-    </row>
-    <row r="6" spans="1:38">
+      <c r="AM5">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="6" spans="1:39">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -2752,8 +3142,11 @@
       <c r="AL6">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:38">
+      <c r="AM6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:39">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -2868,8 +3261,11 @@
       <c r="AL7">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:38">
+      <c r="AM7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:39">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -2984,8 +3380,11 @@
       <c r="AL8">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:38">
+      <c r="AM8">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:39">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -3100,8 +3499,11 @@
       <c r="AL9">
         <v>9</v>
       </c>
-    </row>
-    <row r="10" spans="1:38">
+      <c r="AM9">
+        <v>13.53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:39">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -3216,8 +3618,11 @@
       <c r="AL10">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="11" spans="1:38">
+      <c r="AM10">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:39">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -3331,6 +3736,9 @@
       </c>
       <c r="AL11">
         <v>6</v>
+      </c>
+      <c r="AM11">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3343,13 +3751,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919B50E8-8424-482E-B651-AD901A55E56F}">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -3357,10 +3765,13 @@
         <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+        <v>58</v>
+      </c>
+      <c r="D1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2">
         <v>1995</v>
       </c>
@@ -3370,8 +3781,11 @@
       <c r="C2">
         <v>499.58300000000003</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2">
+        <v>755.05700000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3">
         <v>1995</v>
       </c>
@@ -3381,8 +3795,11 @@
       <c r="C3">
         <v>478.33300000000003</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="D3">
+        <v>748.73599999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>1995</v>
       </c>
@@ -3392,8 +3809,11 @@
       <c r="C4">
         <v>464.16699999999997</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="D4">
+        <v>590.072</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>1995</v>
       </c>
@@ -3403,8 +3823,11 @@
       <c r="C5">
         <v>332.27699999999999</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="D5">
+        <v>508.19299999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>1996</v>
       </c>
@@ -3414,8 +3837,11 @@
       <c r="C6">
         <v>317.16699999999997</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="D6">
+        <v>422.36799999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7">
         <v>1996</v>
       </c>
@@ -3425,8 +3851,11 @@
       <c r="C7">
         <v>324.83300000000003</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="D7">
+        <v>425.29300000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8">
         <v>1996</v>
       </c>
@@ -3436,8 +3865,11 @@
       <c r="C8">
         <v>290</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="D8">
+        <v>354.40100000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9">
         <v>1996</v>
       </c>
@@ -3447,8 +3879,11 @@
       <c r="C9">
         <v>248</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="D9">
+        <v>341.71699999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10">
         <v>1997</v>
       </c>
@@ -3458,8 +3893,11 @@
       <c r="C10">
         <v>260.91699999999997</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="D10">
+        <v>328.964</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11">
         <v>1997</v>
       </c>
@@ -3469,8 +3907,11 @@
       <c r="C11">
         <v>351.66699999999997</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="D11">
+        <v>368.10300000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12">
         <v>1997</v>
       </c>
@@ -3480,8 +3921,11 @@
       <c r="C12">
         <v>375.14</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="D12">
+        <v>408.767</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13">
         <v>1997</v>
       </c>
@@ -3491,8 +3935,11 @@
       <c r="C13">
         <v>383.69299999999998</v>
       </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="D13">
+        <v>449.137</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14">
         <v>1998</v>
       </c>
@@ -3502,8 +3949,11 @@
       <c r="C14">
         <v>437.08300000000003</v>
       </c>
-    </row>
-    <row r="15" spans="1:3">
+      <c r="D14">
+        <v>503.29399999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15">
         <v>1998</v>
       </c>
@@ -3513,8 +3963,11 @@
       <c r="C15">
         <v>359.16699999999997</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
+      <c r="D15">
+        <v>595.99199999999996</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16">
         <v>1998</v>
       </c>
@@ -3524,8 +3977,11 @@
       <c r="C16">
         <v>335.25</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
+      <c r="D16">
+        <v>515.85299999999995</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17">
         <v>1998</v>
       </c>
@@ -3535,8 +3991,11 @@
       <c r="C17">
         <v>408.33300000000003</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
+      <c r="D17">
+        <v>437.32299999999998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18">
         <v>1999</v>
       </c>
@@ -3546,8 +4005,11 @@
       <c r="C18">
         <v>369.81799999999998</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
+      <c r="D18">
+        <v>458.291</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19">
         <v>1999</v>
       </c>
@@ -3557,8 +4019,11 @@
       <c r="C19">
         <v>355.38499999999999</v>
       </c>
-    </row>
-    <row r="20" spans="1:3">
+      <c r="D19">
+        <v>436.238</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20">
         <v>1999</v>
       </c>
@@ -3568,8 +4033,11 @@
       <c r="C20">
         <v>362.30799999999999</v>
       </c>
-    </row>
-    <row r="21" spans="1:3">
+      <c r="D20">
+        <v>467.36099999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21">
         <v>1999</v>
       </c>
@@ -3579,8 +4047,11 @@
       <c r="C21">
         <v>378.23099999999999</v>
       </c>
-    </row>
-    <row r="22" spans="1:3">
+      <c r="D21">
+        <v>452.70499999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22">
         <v>2000</v>
       </c>
@@ -3590,8 +4061,11 @@
       <c r="C22">
         <v>348.46199999999999</v>
       </c>
-    </row>
-    <row r="23" spans="1:3">
+      <c r="D22">
+        <v>441.137</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23">
         <v>2000</v>
       </c>
@@ -3601,8 +4075,11 @@
       <c r="C23">
         <v>396.36399999999998</v>
       </c>
-    </row>
-    <row r="24" spans="1:3">
+      <c r="D23">
+        <v>481.72399999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24">
         <v>2000</v>
       </c>
@@ -3612,8 +4089,11 @@
       <c r="C24">
         <v>410.21600000000001</v>
       </c>
-    </row>
-    <row r="25" spans="1:3">
+      <c r="D24">
+        <v>503.21800000000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25">
         <v>2000</v>
       </c>
@@ -3623,8 +4103,11 @@
       <c r="C25">
         <v>497.25</v>
       </c>
-    </row>
-    <row r="26" spans="1:3">
+      <c r="D25">
+        <v>517.88199999999995</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26">
         <v>2001</v>
       </c>
@@ -3634,8 +4117,11 @@
       <c r="C26">
         <v>552.30799999999999</v>
       </c>
-    </row>
-    <row r="27" spans="1:3">
+      <c r="D26">
+        <v>506.75799999999998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27">
         <v>2001</v>
       </c>
@@ -3645,8 +4131,11 @@
       <c r="C27">
         <v>522.077</v>
       </c>
-    </row>
-    <row r="28" spans="1:3">
+      <c r="D27">
+        <v>608.06100000000004</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28">
         <v>2001</v>
       </c>
@@ -3656,8 +4145,11 @@
       <c r="C28">
         <v>565</v>
       </c>
-    </row>
-    <row r="29" spans="1:3">
+      <c r="D28">
+        <v>637.88699999999994</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29">
         <v>2001</v>
       </c>
@@ -3667,8 +4159,11 @@
       <c r="C29">
         <v>533.21400000000006</v>
       </c>
-    </row>
-    <row r="30" spans="1:3">
+      <c r="D29">
+        <v>592.20100000000002</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30">
         <v>2002</v>
       </c>
@@ -3678,8 +4173,11 @@
       <c r="C30">
         <v>508.75</v>
       </c>
-    </row>
-    <row r="31" spans="1:3">
+      <c r="D30">
+        <v>606.68399999999997</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31">
         <v>2002</v>
       </c>
@@ -3689,8 +4187,11 @@
       <c r="C31">
         <v>520</v>
       </c>
-    </row>
-    <row r="32" spans="1:3">
+      <c r="D31">
+        <v>656.14300000000003</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32">
         <v>2002</v>
       </c>
@@ -3700,8 +4201,11 @@
       <c r="C32">
         <v>520.76900000000001</v>
       </c>
-    </row>
-    <row r="33" spans="1:3">
+      <c r="D32">
+        <v>669.33299999999997</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33">
         <v>2002</v>
       </c>
@@ -3711,8 +4215,11 @@
       <c r="C33">
         <v>522.92899999999997</v>
       </c>
-    </row>
-    <row r="34" spans="1:3">
+      <c r="D33">
+        <v>621.34400000000005</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
       <c r="A34">
         <v>2003</v>
       </c>
@@ -3722,8 +4229,11 @@
       <c r="C34">
         <v>525</v>
       </c>
-    </row>
-    <row r="35" spans="1:3">
+      <c r="D34">
+        <v>586.44100000000003</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
       <c r="A35">
         <v>2003</v>
       </c>
@@ -3733,8 +4243,11 @@
       <c r="C35">
         <v>490.38499999999999</v>
       </c>
-    </row>
-    <row r="36" spans="1:3">
+      <c r="D35">
+        <v>507.59500000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
       <c r="A36">
         <v>2003</v>
       </c>
@@ -3744,8 +4257,11 @@
       <c r="C36">
         <v>437.14299999999997</v>
       </c>
-    </row>
-    <row r="37" spans="1:3">
+      <c r="D36">
+        <v>502.089</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
       <c r="A37">
         <v>2003</v>
       </c>
@@ -3755,8 +4271,11 @@
       <c r="C37">
         <v>359.61500000000001</v>
       </c>
-    </row>
-    <row r="38" spans="1:3">
+      <c r="D37">
+        <v>416.65100000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38">
         <v>2004</v>
       </c>
@@ -3766,8 +4285,11 @@
       <c r="C38">
         <v>310.76900000000001</v>
       </c>
-    </row>
-    <row r="39" spans="1:3">
+      <c r="D38">
+        <v>379.59399999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39">
         <v>2004</v>
       </c>
@@ -3777,8 +4299,11 @@
       <c r="C39">
         <v>323.61500000000001</v>
       </c>
-    </row>
-    <row r="40" spans="1:3">
+      <c r="D39">
+        <v>409.51600000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
       <c r="A40">
         <v>2004</v>
       </c>
@@ -3788,8 +4313,11 @@
       <c r="C40">
         <v>353.69200000000001</v>
       </c>
-    </row>
-    <row r="41" spans="1:3">
+      <c r="D40">
+        <v>430.62099999999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
       <c r="A41">
         <v>2004</v>
       </c>
@@ -3799,8 +4327,11 @@
       <c r="C41">
         <v>326.46199999999999</v>
       </c>
-    </row>
-    <row r="42" spans="1:3">
+      <c r="D41">
+        <v>445.4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
       <c r="A42">
         <v>2005</v>
       </c>
@@ -3810,8 +4341,11 @@
       <c r="C42">
         <v>314.25</v>
       </c>
-    </row>
-    <row r="43" spans="1:3">
+      <c r="D42">
+        <v>410.41800000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
       <c r="A43">
         <v>2005</v>
       </c>
@@ -3821,8 +4355,11 @@
       <c r="C43">
         <v>320</v>
       </c>
-    </row>
-    <row r="44" spans="1:3">
+      <c r="D43">
+        <v>442.81900000000002</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
       <c r="A44">
         <v>2005</v>
       </c>
@@ -3832,8 +4369,11 @@
       <c r="C44">
         <v>320</v>
       </c>
-    </row>
-    <row r="45" spans="1:3">
+      <c r="D44">
+        <v>470.238</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
       <c r="A45">
         <v>2005</v>
       </c>
@@ -3843,8 +4383,11 @@
       <c r="C45">
         <v>363.75</v>
       </c>
-    </row>
-    <row r="46" spans="1:3">
+      <c r="D45">
+        <v>482.24400000000003</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
       <c r="A46">
         <v>2006</v>
       </c>
@@ -3854,8 +4397,11 @@
       <c r="C46">
         <v>394.69200000000001</v>
       </c>
-    </row>
-    <row r="47" spans="1:3">
+      <c r="D46">
+        <v>689.08900000000006</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
       <c r="A47">
         <v>2006</v>
       </c>
@@ -3865,8 +4411,11 @@
       <c r="C47">
         <v>513.846</v>
       </c>
-    </row>
-    <row r="48" spans="1:3">
+      <c r="D47">
+        <v>420.76900000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
       <c r="A48">
         <v>2006</v>
       </c>
@@ -3876,8 +4425,11 @@
       <c r="C48">
         <v>629.23099999999999</v>
       </c>
-    </row>
-    <row r="49" spans="1:3">
+      <c r="D48">
+        <v>688.81899999999996</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
       <c r="A49">
         <v>2006</v>
       </c>
@@ -3887,8 +4439,11 @@
       <c r="C49">
         <v>609.923</v>
       </c>
-    </row>
-    <row r="50" spans="1:3">
+      <c r="D49">
+        <v>673.56100000000004</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
       <c r="A50">
         <v>2007</v>
       </c>
@@ -3898,8 +4453,11 @@
       <c r="C50">
         <v>685.38499999999999</v>
       </c>
-    </row>
-    <row r="51" spans="1:3">
+      <c r="D50">
+        <v>708.23099999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
       <c r="A51">
         <v>2007</v>
       </c>
@@ -3909,8 +4467,11 @@
       <c r="C51">
         <v>687.69200000000001</v>
       </c>
-    </row>
-    <row r="52" spans="1:3">
+      <c r="D51">
+        <v>792.89099999999996</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
       <c r="A52">
         <v>2007</v>
       </c>
@@ -3920,8 +4481,11 @@
       <c r="C52">
         <v>738.46199999999999</v>
       </c>
-    </row>
-    <row r="53" spans="1:3">
+      <c r="D52">
+        <v>892.06399999999996</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
       <c r="A53">
         <v>2007</v>
       </c>
@@ -3931,8 +4495,11 @@
       <c r="C53">
         <v>571.25</v>
       </c>
-    </row>
-    <row r="54" spans="1:3">
+      <c r="D53">
+        <v>633.73900000000003</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
       <c r="A54">
         <v>2008</v>
       </c>
@@ -3942,8 +4509,11 @@
       <c r="C54">
         <v>582.69200000000001</v>
       </c>
-    </row>
-    <row r="55" spans="1:3">
+      <c r="D54">
+        <v>649.50599999999997</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
       <c r="A55">
         <v>2008</v>
       </c>
@@ -3953,8 +4523,11 @@
       <c r="C55">
         <v>698.077</v>
       </c>
-    </row>
-    <row r="56" spans="1:3">
+      <c r="D55">
+        <v>583.45299999999997</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
       <c r="A56">
         <v>2008</v>
       </c>
@@ -3964,8 +4537,11 @@
       <c r="C56">
         <v>702.85699999999997</v>
       </c>
-    </row>
-    <row r="57" spans="1:3">
+      <c r="D56">
+        <v>856.75199999999995</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
       <c r="A57">
         <v>2008</v>
       </c>
@@ -3975,8 +4551,11 @@
       <c r="C57">
         <v>455.90899999999999</v>
       </c>
-    </row>
-    <row r="58" spans="1:3">
+      <c r="D57">
+        <v>610.10199999999998</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
       <c r="A58">
         <v>2009</v>
       </c>
@@ -3986,8 +4565,11 @@
       <c r="C58">
         <v>402.69200000000001</v>
       </c>
-    </row>
-    <row r="59" spans="1:3">
+      <c r="D58">
+        <v>576.43499999999995</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
       <c r="A59">
         <v>2009</v>
       </c>
@@ -3997,8 +4579,11 @@
       <c r="C59">
         <v>446.25</v>
       </c>
-    </row>
-    <row r="60" spans="1:3">
+      <c r="D59">
+        <v>556.71500000000003</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
       <c r="A60">
         <v>2009</v>
       </c>
@@ -4008,8 +4593,11 @@
       <c r="C60">
         <v>455.5</v>
       </c>
-    </row>
-    <row r="61" spans="1:3">
+      <c r="D60">
+        <v>602.21600000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
       <c r="A61">
         <v>2009</v>
       </c>
@@ -4019,8 +4607,11 @@
       <c r="C61">
         <v>433.66699999999997</v>
       </c>
-    </row>
-    <row r="62" spans="1:3">
+      <c r="D61">
+        <v>513.76300000000003</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
       <c r="A62">
         <v>2010</v>
       </c>
@@ -4030,8 +4621,11 @@
       <c r="C62">
         <v>425.46199999999999</v>
       </c>
-    </row>
-    <row r="63" spans="1:3">
+      <c r="D62">
+        <v>570.32600000000002</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
       <c r="A63">
         <v>2010</v>
       </c>
@@ -4041,8 +4635,11 @@
       <c r="C63">
         <v>422.69200000000001</v>
       </c>
-    </row>
-    <row r="64" spans="1:3">
+      <c r="D63">
+        <v>572.851</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
       <c r="A64">
         <v>2010</v>
       </c>
@@ -4052,8 +4649,11 @@
       <c r="C64">
         <v>424</v>
       </c>
-    </row>
-    <row r="65" spans="1:3">
+      <c r="D64">
+        <v>560.19299999999998</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
       <c r="A65">
         <v>2010</v>
       </c>
@@ -4063,8 +4663,11 @@
       <c r="C65">
         <v>464</v>
       </c>
-    </row>
-    <row r="66" spans="1:3">
+      <c r="D65">
+        <v>480.05700000000002</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
       <c r="A66">
         <v>2011</v>
       </c>
@@ -4074,8 +4677,11 @@
       <c r="C66">
         <v>513.58299999999997</v>
       </c>
-    </row>
-    <row r="67" spans="1:3">
+      <c r="D66">
+        <v>535.66800000000001</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
       <c r="A67">
         <v>2011</v>
       </c>
@@ -4085,8 +4691,11 @@
       <c r="C67">
         <v>426.077</v>
       </c>
-    </row>
-    <row r="68" spans="1:3">
+      <c r="D67">
+        <v>518.79899999999998</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
       <c r="A68">
         <v>2011</v>
       </c>
@@ -4096,8 +4705,11 @@
       <c r="C68">
         <v>466.923</v>
       </c>
-    </row>
-    <row r="69" spans="1:3">
+      <c r="D68">
+        <v>523.44600000000003</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
       <c r="A69">
         <v>2011</v>
       </c>
@@ -4107,8 +4719,11 @@
       <c r="C69">
         <v>507.91699999999997</v>
       </c>
-    </row>
-    <row r="70" spans="1:3">
+      <c r="D69">
+        <v>595.505</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
       <c r="A70">
         <v>2012</v>
       </c>
@@ -4118,8 +4733,11 @@
       <c r="C70">
         <v>506.08300000000003</v>
       </c>
-    </row>
-    <row r="71" spans="1:3">
+      <c r="D70">
+        <v>568.95100000000002</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
       <c r="A71">
         <v>2012</v>
       </c>
@@ -4129,8 +4747,11 @@
       <c r="C71">
         <v>618.846</v>
       </c>
-    </row>
-    <row r="72" spans="1:3">
+      <c r="D71">
+        <v>634.33900000000006</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
       <c r="A72">
         <v>2012</v>
       </c>
@@ -4140,8 +4761,11 @@
       <c r="C72">
         <v>639.23099999999999</v>
       </c>
-    </row>
-    <row r="73" spans="1:3">
+      <c r="D72">
+        <v>710.23099999999999</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
       <c r="A73">
         <v>2012</v>
       </c>
@@ -4151,8 +4775,11 @@
       <c r="C73">
         <v>519.61500000000001</v>
       </c>
-    </row>
-    <row r="74" spans="1:3">
+      <c r="D73">
+        <v>623.33900000000006</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
       <c r="A74">
         <v>2013</v>
       </c>
@@ -4162,8 +4789,11 @@
       <c r="C74">
         <v>519.16700000000003</v>
       </c>
-    </row>
-    <row r="75" spans="1:3">
+      <c r="D74">
+        <v>594.83699999999999</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
       <c r="A75">
         <v>2013</v>
       </c>
@@ -4173,8 +4803,11 @@
       <c r="C75">
         <v>526.53800000000001</v>
       </c>
-    </row>
-    <row r="76" spans="1:3">
+      <c r="D75">
+        <v>612.47400000000005</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
       <c r="A76">
         <v>2013</v>
       </c>
@@ -4184,8 +4817,11 @@
       <c r="C76">
         <v>431.07100000000003</v>
       </c>
-    </row>
-    <row r="77" spans="1:3">
+      <c r="D76">
+        <v>619.88599999999997</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
       <c r="A77">
         <v>2013</v>
       </c>
@@ -4195,8 +4831,11 @@
       <c r="C77">
         <v>398.63600000000002</v>
       </c>
-    </row>
-    <row r="78" spans="1:3">
+      <c r="D77">
+        <v>498.399</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
       <c r="A78">
         <v>2014</v>
       </c>
@@ -4206,8 +4845,11 @@
       <c r="C78">
         <v>453.46199999999999</v>
       </c>
-    </row>
-    <row r="79" spans="1:3">
+      <c r="D78">
+        <v>536.50300000000004</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
       <c r="A79">
         <v>2014</v>
       </c>
@@ -4217,8 +4859,11 @@
       <c r="C79">
         <v>456.53800000000001</v>
       </c>
-    </row>
-    <row r="80" spans="1:3">
+      <c r="D79">
+        <v>534.13599999999997</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
       <c r="A80">
         <v>2014</v>
       </c>
@@ -4228,8 +4873,11 @@
       <c r="C80">
         <v>446.154</v>
       </c>
-    </row>
-    <row r="81" spans="1:3">
+      <c r="D80">
+        <v>556.37099999999998</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
       <c r="A81">
         <v>2014</v>
       </c>
@@ -4239,8 +4887,11 @@
       <c r="C81">
         <v>460.45499999999998</v>
       </c>
-    </row>
-    <row r="82" spans="1:3">
+      <c r="D81">
+        <v>570.94100000000003</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
       <c r="A82">
         <v>2015</v>
       </c>
@@ -4250,8 +4901,11 @@
       <c r="C82">
         <v>606.53800000000001</v>
       </c>
-    </row>
-    <row r="83" spans="1:3">
+      <c r="D82">
+        <v>618.13400000000001</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
       <c r="A83">
         <v>2015</v>
       </c>
@@ -4261,8 +4915,11 @@
       <c r="C83">
         <v>784.23099999999999</v>
       </c>
-    </row>
-    <row r="84" spans="1:3">
+      <c r="D83">
+        <v>699.31700000000001</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
       <c r="A84">
         <v>2015</v>
       </c>
@@ -4272,8 +4929,11 @@
       <c r="C84">
         <v>830.38499999999999</v>
       </c>
-    </row>
-    <row r="85" spans="1:3">
+      <c r="D84">
+        <v>874.28599999999994</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
       <c r="A85">
         <v>2015</v>
       </c>
@@ -4283,8 +4943,11 @@
       <c r="C85">
         <v>806.66700000000003</v>
       </c>
-    </row>
-    <row r="86" spans="1:3">
+      <c r="D85">
+        <v>865.18200000000002</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
       <c r="A86">
         <v>2016</v>
       </c>
@@ -4294,8 +4957,11 @@
       <c r="C86">
         <v>1004.167</v>
       </c>
-    </row>
-    <row r="87" spans="1:3">
+      <c r="D86">
+        <v>903.51599999999996</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
       <c r="A87">
         <v>2016</v>
       </c>
@@ -4305,8 +4971,11 @@
       <c r="C87">
         <v>1137.692</v>
       </c>
-    </row>
-    <row r="88" spans="1:3">
+      <c r="D87">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
       <c r="A88">
         <v>2016</v>
       </c>
@@ -4316,8 +4985,11 @@
       <c r="C88">
         <v>1120.385</v>
       </c>
-    </row>
-    <row r="89" spans="1:3">
+      <c r="D88">
+        <v>1272.3209999999999</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
       <c r="A89">
         <v>2016</v>
       </c>
@@ -4327,8 +4999,11 @@
       <c r="C89">
         <v>797.08299999999997</v>
       </c>
-    </row>
-    <row r="90" spans="1:3">
+      <c r="D89">
+        <v>968.21</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
       <c r="A90">
         <v>2017</v>
       </c>
@@ -4338,8 +5013,11 @@
       <c r="C90">
         <v>847.08299999999997</v>
       </c>
-    </row>
-    <row r="91" spans="1:3">
+      <c r="D90">
+        <v>941.61800000000005</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
       <c r="A91">
         <v>2017</v>
       </c>
@@ -4349,8 +5027,11 @@
       <c r="C91">
         <v>1018.462</v>
       </c>
-    </row>
-    <row r="92" spans="1:3">
+      <c r="D91">
+        <v>1024.4010000000001</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
       <c r="A92">
         <v>2017</v>
       </c>
@@ -4360,8 +5041,11 @@
       <c r="C92">
         <v>867.69200000000001</v>
       </c>
-    </row>
-    <row r="93" spans="1:3">
+      <c r="D92">
+        <v>1012.489</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
       <c r="A93">
         <v>2017</v>
       </c>
@@ -4371,8 +5055,11 @@
       <c r="C93">
         <v>757.5</v>
       </c>
-    </row>
-    <row r="94" spans="1:3">
+      <c r="D93">
+        <v>956.71500000000003</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
       <c r="A94">
         <v>2018</v>
       </c>
@@ -4382,8 +5069,11 @@
       <c r="C94">
         <v>615.83299999999997</v>
       </c>
-    </row>
-    <row r="95" spans="1:3">
+      <c r="D94">
+        <v>820.97</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
       <c r="A95">
         <v>2018</v>
       </c>
@@ -4393,8 +5083,11 @@
       <c r="C95">
         <v>625.38499999999999</v>
       </c>
-    </row>
-    <row r="96" spans="1:3">
+      <c r="D95">
+        <v>737.44500000000005</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
       <c r="A96">
         <v>2018</v>
       </c>
@@ -4404,8 +5097,11 @@
       <c r="C96">
         <v>743.46199999999999</v>
       </c>
-    </row>
-    <row r="97" spans="1:3">
+      <c r="D96">
+        <v>764.09</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
       <c r="A97">
         <v>2018</v>
       </c>
@@ -4415,8 +5111,11 @@
       <c r="C97">
         <v>803.92899999999997</v>
       </c>
-    </row>
-    <row r="98" spans="1:3">
+      <c r="D97">
+        <v>834.80499999999995</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
       <c r="A98">
         <v>2019</v>
       </c>
@@ -4426,8 +5125,11 @@
       <c r="C98">
         <v>797.5</v>
       </c>
-    </row>
-    <row r="99" spans="1:3">
+      <c r="D98">
+        <v>896.34699999999998</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4">
       <c r="A99">
         <v>2019</v>
       </c>
@@ -4437,8 +5139,11 @@
       <c r="C99">
         <v>696.69200000000001</v>
       </c>
-    </row>
-    <row r="100" spans="1:3">
+      <c r="D99">
+        <v>837.12099999999998</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4">
       <c r="A100">
         <v>2019</v>
       </c>
@@ -4448,8 +5153,11 @@
       <c r="C100">
         <v>650.71400000000006</v>
       </c>
-    </row>
-    <row r="101" spans="1:3">
+      <c r="D100">
+        <v>749.08699999999999</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
       <c r="A101">
         <v>2019</v>
       </c>
@@ -4459,8 +5167,11 @@
       <c r="C101">
         <v>777.5</v>
       </c>
-    </row>
-    <row r="102" spans="1:3">
+      <c r="D101">
+        <v>829.52200000000005</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4">
       <c r="A102">
         <v>2020</v>
       </c>
@@ -4470,8 +5181,11 @@
       <c r="C102">
         <v>855.76900000000001</v>
       </c>
-    </row>
-    <row r="103" spans="1:3">
+      <c r="D102">
+        <v>855.56100000000004</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4">
       <c r="A103">
         <v>2020</v>
       </c>
@@ -4481,8 +5195,11 @@
       <c r="C103">
         <v>735.923</v>
       </c>
-    </row>
-    <row r="104" spans="1:3">
+      <c r="D103">
+        <v>866.63099999999997</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4">
       <c r="A104">
         <v>2020</v>
       </c>
@@ -4492,8 +5209,11 @@
       <c r="C104">
         <v>627.69200000000001</v>
       </c>
-    </row>
-    <row r="105" spans="1:3">
+      <c r="D104">
+        <v>771.02</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4">
       <c r="A105">
         <v>2020</v>
       </c>
@@ -4503,8 +5223,11 @@
       <c r="C105">
         <v>582.53800000000001</v>
       </c>
-    </row>
-    <row r="106" spans="1:3">
+      <c r="D105">
+        <v>693.18600000000004</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4">
       <c r="A106">
         <v>2021</v>
       </c>
@@ -4514,8 +5237,11 @@
       <c r="C106">
         <v>616.154</v>
       </c>
-    </row>
-    <row r="107" spans="1:3">
+      <c r="D106">
+        <v>691.71799999999996</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4">
       <c r="A107">
         <v>2021</v>
       </c>
@@ -4525,8 +5251,11 @@
       <c r="C107">
         <v>679.23099999999999</v>
       </c>
-    </row>
-    <row r="108" spans="1:3">
+      <c r="D107">
+        <v>751.46799999999996</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4">
       <c r="A108">
         <v>2021</v>
       </c>
@@ -4536,8 +5265,11 @@
       <c r="C108">
         <v>615.76900000000001</v>
       </c>
-    </row>
-    <row r="109" spans="1:3">
+      <c r="D108">
+        <v>757.40300000000002</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4">
       <c r="A109">
         <v>2021</v>
       </c>
@@ -4547,8 +5279,11 @@
       <c r="C109">
         <v>549.61500000000001</v>
       </c>
-    </row>
-    <row r="110" spans="1:3">
+      <c r="D109">
+        <v>794.33399999999995</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4">
       <c r="A110">
         <v>2022</v>
       </c>
@@ -4558,8 +5293,11 @@
       <c r="C110">
         <v>550.76900000000001</v>
       </c>
-    </row>
-    <row r="111" spans="1:3">
+      <c r="D110">
+        <v>771.42600000000004</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4">
       <c r="A111">
         <v>2022</v>
       </c>
@@ -4569,8 +5307,11 @@
       <c r="C111">
         <v>533.923</v>
       </c>
-    </row>
-    <row r="112" spans="1:3">
+      <c r="D111">
+        <v>861.61500000000001</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4">
       <c r="A112">
         <v>2022</v>
       </c>
@@ -4580,8 +5321,11 @@
       <c r="C112">
         <v>549.23099999999999</v>
       </c>
-    </row>
-    <row r="113" spans="1:3">
+      <c r="D112">
+        <v>902.09699999999998</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4">
       <c r="A113">
         <v>2022</v>
       </c>
@@ -4591,8 +5335,11 @@
       <c r="C113">
         <v>532.5</v>
       </c>
-    </row>
-    <row r="114" spans="1:3">
+      <c r="D113">
+        <v>786.10599999999999</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4">
       <c r="A114">
         <v>2023</v>
       </c>
@@ -4602,8 +5349,11 @@
       <c r="C114">
         <v>576.53800000000001</v>
       </c>
-    </row>
-    <row r="115" spans="1:3">
+      <c r="D114">
+        <v>811.37099999999998</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4">
       <c r="A115">
         <v>2023</v>
       </c>
@@ -4613,8 +5363,11 @@
       <c r="C115">
         <v>596.66700000000003</v>
       </c>
-    </row>
-    <row r="116" spans="1:3">
+      <c r="D115">
+        <v>769.43100000000004</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4">
       <c r="A116">
         <v>2023</v>
       </c>
@@ -4624,8 +5377,11 @@
       <c r="C116">
         <v>691.53800000000001</v>
       </c>
-    </row>
-    <row r="117" spans="1:3">
+      <c r="D116">
+        <v>663.26300000000003</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
       <c r="A117">
         <v>2023</v>
       </c>
@@ -4635,8 +5391,11 @@
       <c r="C117">
         <v>822.5</v>
       </c>
-    </row>
-    <row r="118" spans="1:3">
+      <c r="D117">
+        <v>839.178</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4">
       <c r="A118">
         <v>2024</v>
       </c>
@@ -4646,8 +5405,11 @@
       <c r="C118">
         <v>870.76900000000001</v>
       </c>
-    </row>
-    <row r="119" spans="1:3">
+      <c r="D118">
+        <v>965.32899999999995</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4">
       <c r="A119">
         <v>2024</v>
       </c>
@@ -4657,8 +5419,11 @@
       <c r="C119">
         <v>943.846</v>
       </c>
-    </row>
-    <row r="120" spans="1:3">
+      <c r="D119">
+        <v>1022.404</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4">
       <c r="A120">
         <v>2024</v>
       </c>
@@ -4668,8 +5433,11 @@
       <c r="C120">
         <v>965.71400000000006</v>
       </c>
-    </row>
-    <row r="121" spans="1:3">
+      <c r="D120">
+        <v>1073.9680000000001</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4">
       <c r="A121">
         <v>2024</v>
       </c>
@@ -4678,6 +5446,51 @@
       </c>
       <c r="C121">
         <v>902.30799999999999</v>
+      </c>
+      <c r="D121">
+        <v>1082.2</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4">
+      <c r="A122">
+        <v>2025</v>
+      </c>
+      <c r="B122" t="s">
+        <v>53</v>
+      </c>
+      <c r="C122">
+        <v>938.75</v>
+      </c>
+      <c r="D122">
+        <v>898.76900000000001</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4">
+      <c r="A123">
+        <v>2025</v>
+      </c>
+      <c r="B123" t="s">
+        <v>50</v>
+      </c>
+      <c r="C123">
+        <v>913.846</v>
+      </c>
+      <c r="D123">
+        <v>1027.239</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4">
+      <c r="A124">
+        <v>2025</v>
+      </c>
+      <c r="B124" t="s">
+        <v>51</v>
+      </c>
+      <c r="C124">
+        <v>797.69200000000001</v>
+      </c>
+      <c r="D124">
+        <v>901.85199999999998</v>
       </c>
     </row>
   </sheetData>
@@ -4690,15 +5503,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8E49554-F216-4D4D-8656-92A00E89040E}">
-  <dimension ref="A1:E37"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9D1B0BF-D15E-4BA5-969C-124619CD39F7}">
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.44140625" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>44</v>
       </c>
@@ -4714,8 +5527,868 @@
       <c r="E1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>95.433999999999997</v>
+      </c>
+      <c r="D2">
+        <v>67.546999999999997</v>
+      </c>
+      <c r="E2">
+        <v>85.971000000000004</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3">
+        <v>446.65300000000002</v>
+      </c>
+      <c r="C3">
+        <v>85.72</v>
+      </c>
+      <c r="D3">
+        <v>93.078999999999994</v>
+      </c>
+      <c r="E3">
+        <v>109.36799999999999</v>
+      </c>
+      <c r="F3">
+        <v>48.85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4">
+        <v>229.56399999999999</v>
+      </c>
+      <c r="C4">
+        <v>147.35900000000001</v>
+      </c>
+      <c r="D4">
+        <v>178.12100000000001</v>
+      </c>
+      <c r="E4">
+        <v>191.66800000000001</v>
+      </c>
+      <c r="F4">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5">
+        <v>250.583</v>
+      </c>
+      <c r="C5">
+        <v>86.367000000000004</v>
+      </c>
+      <c r="D5">
+        <v>249.672</v>
+      </c>
+      <c r="E5">
+        <v>221.85900000000001</v>
+      </c>
+      <c r="F5">
+        <v>55.594000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6">
+        <v>292.47300000000001</v>
+      </c>
+      <c r="C6">
+        <v>228.458</v>
+      </c>
+      <c r="D6">
+        <v>151.80199999999999</v>
+      </c>
+      <c r="E6">
+        <v>176.93799999999999</v>
+      </c>
+      <c r="F6">
+        <v>51.75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7">
+        <v>375.286</v>
+      </c>
+      <c r="C7">
+        <v>222.14500000000001</v>
+      </c>
+      <c r="D7">
+        <v>146.83699999999999</v>
+      </c>
+      <c r="E7">
+        <v>193.108</v>
+      </c>
+      <c r="F7">
+        <v>72.471000000000004</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8">
+        <v>495.91</v>
+      </c>
+      <c r="C8">
+        <v>36.463999999999999</v>
+      </c>
+      <c r="D8">
+        <v>208.85400000000001</v>
+      </c>
+      <c r="E8">
+        <v>68.893000000000001</v>
+      </c>
+      <c r="F8">
+        <v>34.164999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9">
+        <v>365.40199999999999</v>
+      </c>
+      <c r="C9">
+        <v>112.67</v>
+      </c>
+      <c r="D9">
+        <v>216.41499999999999</v>
+      </c>
+      <c r="E9">
+        <v>286.90899999999999</v>
+      </c>
+      <c r="F9">
+        <v>104.837</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10">
+        <v>277.21800000000002</v>
+      </c>
+      <c r="C10">
+        <v>341.85899999999998</v>
+      </c>
+      <c r="D10">
+        <v>241.45</v>
+      </c>
+      <c r="E10">
+        <v>287.721</v>
+      </c>
+      <c r="F10">
+        <v>79.760999999999996</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11">
+        <v>375.34699999999998</v>
+      </c>
+      <c r="C11">
+        <v>255.875</v>
+      </c>
+      <c r="D11">
+        <v>273.04300000000001</v>
+      </c>
+      <c r="E11">
+        <v>198.62899999999999</v>
+      </c>
+      <c r="F11">
+        <v>74.555000000000007</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12">
+        <v>382.82499999999999</v>
+      </c>
+      <c r="C12">
+        <v>109.633</v>
+      </c>
+      <c r="D12">
+        <v>308.505</v>
+      </c>
+      <c r="E12">
+        <v>187.58699999999999</v>
+      </c>
+      <c r="F12">
+        <v>71.813000000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13">
+        <v>339.37</v>
+      </c>
+      <c r="C13">
+        <v>217.69900000000001</v>
+      </c>
+      <c r="D13">
+        <v>217.95500000000001</v>
+      </c>
+      <c r="E13">
+        <v>230.00700000000001</v>
+      </c>
+      <c r="F13">
+        <v>78.058000000000007</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14">
+        <v>462.95100000000002</v>
+      </c>
+      <c r="C14">
+        <v>217.85499999999999</v>
+      </c>
+      <c r="D14">
+        <v>261.60300000000001</v>
+      </c>
+      <c r="E14">
+        <v>162.49199999999999</v>
+      </c>
+      <c r="F14">
+        <v>75.225999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15">
+        <v>475.97699999999998</v>
+      </c>
+      <c r="C15">
+        <v>278.27199999999999</v>
+      </c>
+      <c r="D15">
+        <v>244.93600000000001</v>
+      </c>
+      <c r="E15">
+        <v>273.43900000000002</v>
+      </c>
+      <c r="F15">
+        <v>130.15100000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16">
+        <v>485.75900000000001</v>
+      </c>
+      <c r="C16">
+        <v>88.537999999999997</v>
+      </c>
+      <c r="D16">
+        <v>201.161</v>
+      </c>
+      <c r="E16">
+        <v>128.738</v>
+      </c>
+      <c r="F16">
+        <v>62.536000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>309.17200000000003</v>
+      </c>
+      <c r="C17">
+        <v>163.75299999999999</v>
+      </c>
+      <c r="D17">
+        <v>200.815</v>
+      </c>
+      <c r="E17">
+        <v>198.85400000000001</v>
+      </c>
+      <c r="F17">
+        <v>61.48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>266.553</v>
+      </c>
+      <c r="C18">
+        <v>151.19900000000001</v>
+      </c>
+      <c r="D18">
+        <v>110.17400000000001</v>
+      </c>
+      <c r="E18">
+        <v>135.215</v>
+      </c>
+      <c r="F18">
+        <v>36.042000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>374.40199999999999</v>
+      </c>
+      <c r="C19">
+        <v>211.36099999999999</v>
+      </c>
+      <c r="D19">
+        <v>131.30099999999999</v>
+      </c>
+      <c r="E19">
+        <v>149.68199999999999</v>
+      </c>
+      <c r="F19">
+        <v>56.040999999999997</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>598.14499999999998</v>
+      </c>
+      <c r="C20">
+        <v>244.08099999999999</v>
+      </c>
+      <c r="D20">
+        <v>284.07400000000001</v>
+      </c>
+      <c r="E20">
+        <v>229.202</v>
+      </c>
+      <c r="F20">
+        <v>137.096</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21">
+        <v>621.56399999999996</v>
+      </c>
+      <c r="C21">
+        <v>218.345</v>
+      </c>
+      <c r="D21">
+        <v>306</v>
+      </c>
+      <c r="E21">
+        <v>312.95</v>
+      </c>
+      <c r="F21">
+        <v>194.518</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22">
+        <v>450.00700000000001</v>
+      </c>
+      <c r="C22">
+        <v>466.49599999999998</v>
+      </c>
+      <c r="D22">
+        <v>338.22199999999998</v>
+      </c>
+      <c r="E22">
+        <v>442.54300000000001</v>
+      </c>
+      <c r="F22">
+        <v>199.14699999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23">
+        <v>443.17599999999999</v>
+      </c>
+      <c r="C23">
+        <v>458.81799999999998</v>
+      </c>
+      <c r="D23">
+        <v>428.98200000000003</v>
+      </c>
+      <c r="E23">
+        <v>487.04599999999999</v>
+      </c>
+      <c r="F23">
+        <v>215.84700000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24">
+        <v>403.983</v>
+      </c>
+      <c r="C24">
+        <v>409.13400000000001</v>
+      </c>
+      <c r="D24">
+        <v>653.14200000000005</v>
+      </c>
+      <c r="E24">
+        <v>513.38800000000003</v>
+      </c>
+      <c r="F24">
+        <v>207.4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25">
+        <v>456.65699999999998</v>
+      </c>
+      <c r="C25">
+        <v>652.846</v>
+      </c>
+      <c r="D25">
+        <v>456.07</v>
+      </c>
+      <c r="E25">
+        <v>673.37199999999996</v>
+      </c>
+      <c r="F25">
+        <v>307.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26">
+        <v>393.53300000000002</v>
+      </c>
+      <c r="C26">
+        <v>852.08699999999999</v>
+      </c>
+      <c r="D26">
+        <v>573.6</v>
+      </c>
+      <c r="E26">
+        <v>813.3</v>
+      </c>
+      <c r="F26">
+        <v>320.06</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27">
+        <v>352.28100000000001</v>
+      </c>
+      <c r="C27">
+        <v>561.93499999999995</v>
+      </c>
+      <c r="D27">
+        <v>507.8</v>
+      </c>
+      <c r="E27">
+        <v>629.4</v>
+      </c>
+      <c r="F27">
+        <v>221.726</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28">
+        <v>566.54499999999996</v>
+      </c>
+      <c r="C28">
+        <v>673.84500000000003</v>
+      </c>
+      <c r="D28">
+        <v>424.8</v>
+      </c>
+      <c r="E28">
+        <v>555.4</v>
+      </c>
+      <c r="F28">
+        <v>314.65899999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>41</v>
+      </c>
+      <c r="B29">
+        <v>783.56100000000004</v>
+      </c>
+      <c r="C29">
+        <v>1140.088</v>
+      </c>
+      <c r="D29">
+        <v>677.44399999999996</v>
+      </c>
+      <c r="E29">
+        <v>874.59299999999996</v>
+      </c>
+      <c r="F29">
+        <v>685.298</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30">
+        <v>832.61400000000003</v>
+      </c>
+      <c r="C30">
+        <v>1969.9639999999999</v>
+      </c>
+      <c r="D30">
+        <v>1069</v>
+      </c>
+      <c r="E30">
+        <v>2004</v>
+      </c>
+      <c r="F30">
+        <v>1668.559</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31">
+        <v>651.35900000000004</v>
+      </c>
+      <c r="C31">
+        <v>1135.367</v>
+      </c>
+      <c r="D31">
+        <v>1075.136</v>
+      </c>
+      <c r="E31">
+        <v>998.23099999999999</v>
+      </c>
+      <c r="F31">
+        <v>650.20600000000002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>24</v>
+      </c>
+      <c r="B32">
+        <v>1126.117</v>
+      </c>
+      <c r="C32">
+        <v>335.33100000000002</v>
+      </c>
+      <c r="D32">
+        <v>293.947</v>
+      </c>
+      <c r="E32">
+        <v>205.13</v>
+      </c>
+      <c r="F32">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>22</v>
+      </c>
+      <c r="B33">
+        <v>760.78099999999995</v>
+      </c>
+      <c r="C33">
+        <v>370.23399999999998</v>
+      </c>
+      <c r="D33">
+        <v>309.15100000000001</v>
+      </c>
+      <c r="E33">
+        <v>235.16499999999999</v>
+      </c>
+      <c r="F33">
+        <v>178.90899999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34">
+        <v>592.98299999999995</v>
+      </c>
+      <c r="C34">
+        <v>764.721</v>
+      </c>
+      <c r="D34">
+        <v>606.31600000000003</v>
+      </c>
+      <c r="E34">
+        <v>876.46799999999996</v>
+      </c>
+      <c r="F34">
+        <v>519.73099999999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35">
+        <v>683.28300000000002</v>
+      </c>
+      <c r="C35">
+        <v>605.40300000000002</v>
+      </c>
+      <c r="D35">
+        <v>615.75</v>
+      </c>
+      <c r="E35">
+        <v>1062.25</v>
+      </c>
+      <c r="F35">
+        <v>725.81700000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>46</v>
+      </c>
+      <c r="B36">
+        <v>626.05999999999995</v>
+      </c>
+      <c r="C36">
+        <v>676.42</v>
+      </c>
+      <c r="D36">
+        <v>397.5</v>
+      </c>
+      <c r="E36">
+        <v>541</v>
+      </c>
+      <c r="F36">
+        <v>338.69900000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37">
+        <v>734.63300000000004</v>
+      </c>
+      <c r="C37">
+        <v>606.69200000000001</v>
+      </c>
+      <c r="D37">
+        <v>409</v>
+      </c>
+      <c r="E37">
+        <v>491.2</v>
+      </c>
+      <c r="F37">
+        <v>360.85199999999998</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>49</v>
+      </c>
+      <c r="B38">
+        <v>846.3</v>
+      </c>
+      <c r="C38">
+        <v>2050.3530000000001</v>
+      </c>
+      <c r="D38">
+        <v>1038.5</v>
+      </c>
+      <c r="E38">
+        <v>2267</v>
+      </c>
+      <c r="F38">
+        <v>1918.5619999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" t="s">
+        <v>57</v>
+      </c>
+      <c r="B39">
+        <v>645.16099999999994</v>
+      </c>
+      <c r="C39">
+        <v>1714.365</v>
+      </c>
+      <c r="D39">
+        <v>1083.5</v>
+      </c>
+      <c r="E39">
+        <v>2119.5300000000002</v>
+      </c>
+      <c r="F39">
+        <v>1367.4380000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="10"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="31" type="noConversion"/>
+  <conditionalFormatting sqref="D2:D39">
+    <cfRule type="cellIs" dxfId="40" priority="11" stopIfTrue="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="39" priority="12" stopIfTrue="1" operator="lessThanOrEqual">
+      <formula>-100</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="13" stopIfTrue="1" operator="between">
+      <formula>-99.999999999999</formula>
+      <formula>99.999999999999</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="14" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F39">
+    <cfRule type="cellIs" dxfId="32" priority="7" stopIfTrue="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="31" priority="8" stopIfTrue="1" operator="lessThanOrEqual">
+      <formula>-100</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="9" stopIfTrue="1" operator="between">
+      <formula>-99.999999999999</formula>
+      <formula>99.999999999999</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="10" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E39">
+    <cfRule type="cellIs" dxfId="24" priority="3" stopIfTrue="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="23" priority="4" stopIfTrue="1" operator="lessThanOrEqual">
+      <formula>-100</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="5" stopIfTrue="1" operator="between">
+      <formula>-99.999999999999</formula>
+      <formula>99.999999999999</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="6" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B37">
+    <cfRule type="cellIs" dxfId="18" priority="1" operator="lessThanOrEqual">
+      <formula>99.9999999999</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="17" priority="2" operator="greaterThanOrEqual">
+      <formula>100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8E49554-F216-4D4D-8656-92A00E89040E}">
+  <dimension ref="A1:F39"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -4731,8 +6404,11 @@
       <c r="E2">
         <v>109.36799999999999</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2">
+        <v>48.85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -4748,8 +6424,11 @@
       <c r="E3">
         <v>191.66800000000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -4765,8 +6444,11 @@
       <c r="E4">
         <v>221.85900000000001</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4">
+        <v>55.594000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -4782,8 +6464,11 @@
       <c r="E5">
         <v>176.93799999999999</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="F5">
+        <v>51.75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -4799,8 +6484,11 @@
       <c r="E6">
         <v>193.108</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="F6">
+        <v>72.471000000000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -4816,8 +6504,11 @@
       <c r="E7">
         <v>68.893000000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="F7">
+        <v>34.164999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -4833,8 +6524,11 @@
       <c r="E8">
         <v>286.90899999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="F8">
+        <v>104.837</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -4850,8 +6544,11 @@
       <c r="E9">
         <v>287.721</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="F9">
+        <v>79.760999999999996</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -4867,8 +6564,11 @@
       <c r="E10">
         <v>198.62899999999999</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="F10">
+        <v>74.555000000000007</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>34</v>
       </c>
@@ -4884,8 +6584,11 @@
       <c r="E11">
         <v>187.58699999999999</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="F11">
+        <v>71.813000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -4901,8 +6604,11 @@
       <c r="E12">
         <v>230.00700000000001</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="F12">
+        <v>78.058000000000007</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -4918,8 +6624,11 @@
       <c r="E13">
         <v>162.49199999999999</v>
       </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="F13">
+        <v>75.225999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -4935,8 +6644,11 @@
       <c r="E14">
         <v>273.43900000000002</v>
       </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="F14">
+        <v>130.15100000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>38</v>
       </c>
@@ -4952,8 +6664,11 @@
       <c r="E15">
         <v>128.738</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="F15">
+        <v>62.536000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -4969,8 +6684,11 @@
       <c r="E16">
         <v>198.85400000000001</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="F16">
+        <v>61.48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -4986,8 +6704,11 @@
       <c r="E17">
         <v>135.215</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="F17">
+        <v>36.042000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -5003,8 +6724,11 @@
       <c r="E18">
         <v>149.68199999999999</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="F18">
+        <v>56.040999999999997</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -5020,8 +6744,11 @@
       <c r="E19">
         <v>229.202</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="F19">
+        <v>137.096</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -5037,8 +6764,11 @@
       <c r="E20">
         <v>312.95</v>
       </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="F20">
+        <v>194.518</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -5054,8 +6784,11 @@
       <c r="E21">
         <v>442.54300000000001</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="F21">
+        <v>199.14699999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -5071,8 +6804,11 @@
       <c r="E22">
         <v>487.04599999999999</v>
       </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="F22">
+        <v>215.84700000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>5</v>
       </c>
@@ -5088,8 +6824,11 @@
       <c r="E23">
         <v>513.38800000000003</v>
       </c>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="F23">
+        <v>207.4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>39</v>
       </c>
@@ -5105,8 +6844,11 @@
       <c r="E24">
         <v>673.37199999999996</v>
       </c>
-    </row>
-    <row r="25" spans="1:5">
+      <c r="F24">
+        <v>307.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>40</v>
       </c>
@@ -5122,8 +6864,11 @@
       <c r="E25">
         <v>813.3</v>
       </c>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="F25">
+        <v>320.06</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>6</v>
       </c>
@@ -5139,8 +6884,11 @@
       <c r="E26">
         <v>629.4</v>
       </c>
-    </row>
-    <row r="27" spans="1:5">
+      <c r="F26">
+        <v>221.726</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>7</v>
       </c>
@@ -5156,8 +6904,11 @@
       <c r="E27">
         <v>555.4</v>
       </c>
-    </row>
-    <row r="28" spans="1:5">
+      <c r="F27">
+        <v>314.65899999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>41</v>
       </c>
@@ -5173,8 +6924,11 @@
       <c r="E28">
         <v>874.59299999999996</v>
       </c>
-    </row>
-    <row r="29" spans="1:5">
+      <c r="F28">
+        <v>685.298</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -5190,8 +6944,11 @@
       <c r="E29">
         <v>2004</v>
       </c>
-    </row>
-    <row r="30" spans="1:5">
+      <c r="F29">
+        <v>1668.559</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -5207,8 +6964,11 @@
       <c r="E30">
         <v>998.23099999999999</v>
       </c>
-    </row>
-    <row r="31" spans="1:5">
+      <c r="F30">
+        <v>650.20600000000002</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>24</v>
       </c>
@@ -5224,8 +6984,11 @@
       <c r="E31">
         <v>205.13</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="F31">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -5241,8 +7004,11 @@
       <c r="E32">
         <v>235.16499999999999</v>
       </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="F32">
+        <v>178.90899999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>43</v>
       </c>
@@ -5258,8 +7024,11 @@
       <c r="E33">
         <v>876.46799999999996</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="F33">
+        <v>519.73099999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>48</v>
       </c>
@@ -5275,8 +7044,11 @@
       <c r="E34">
         <v>1062.25</v>
       </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="F34">
+        <v>725.81700000000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>46</v>
       </c>
@@ -5292,13 +7064,16 @@
       <c r="E35">
         <v>541</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="F35">
+        <v>338.69900000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>47</v>
       </c>
       <c r="B36">
-        <v>795.80700000000002</v>
+        <v>734.63300000000004</v>
       </c>
       <c r="D36">
         <v>409</v>
@@ -5306,13 +7081,16 @@
       <c r="E36">
         <v>491.2</v>
       </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="F36">
+        <v>360.85199999999998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="2">
-        <v>937.28933333333327</v>
+      <c r="B37">
+        <v>846.3</v>
       </c>
       <c r="D37">
         <v>1038.5</v>
@@ -5320,6 +7098,32 @@
       <c r="E37">
         <v>2267</v>
       </c>
+      <c r="F37">
+        <v>1918.5619999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>57</v>
+      </c>
+      <c r="B38">
+        <v>645.16099999999994</v>
+      </c>
+      <c r="D38">
+        <v>1083.5</v>
+      </c>
+      <c r="E38">
+        <v>2120</v>
+      </c>
+      <c r="F38">
+        <v>1367.4380000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="10"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="31" type="noConversion"/>
@@ -5330,7 +7134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C756E14-1818-4D47-8560-4E8F304FA0A2}">
   <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6090,7 +7894,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36D69D08-A1A2-4712-9861-8AB21AFF4582}">
   <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6850,7 +8654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E23DAC47-F5FC-4440-BAA8-19C4DEAADCE9}">
   <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7632,20 +9436,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="1f3c66e0-7684-4412-85ae-938bcfc42664" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1f3c66e0-7684-4412-85ae-938bcfc42664">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9c30d4e8-d9db-43d6-83e2-c08e4749ca29" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B8E840779CD5394DB6A0677C69D57CD3" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3a115b2da8a2eeee135fdd5733988381">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="1f3c66e0-7684-4412-85ae-938bcfc42664" xmlns:ns3="9c30d4e8-d9db-43d6-83e2-c08e4749ca29" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="46fe6ebd3e8bf6d9df49fa3e9a691e0f" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -7905,6 +9695,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="1f3c66e0-7684-4412-85ae-938bcfc42664" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1f3c66e0-7684-4412-85ae-938bcfc42664">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9c30d4e8-d9db-43d6-83e2-c08e4749ca29" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA51C66A-940B-4EBF-AB7C-C7E573134CC8}">
   <ds:schemaRefs>
@@ -7914,24 +9718,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60AF7E67-B0A8-4403-B034-291A80FBDDB1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9c30d4e8-d9db-43d6-83e2-c08e4749ca29"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1f3c66e0-7684-4412-85ae-938bcfc42664"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C17C4D53-3825-44BD-9FD0-63343C204D24}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7951,6 +9737,24 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60AF7E67-B0A8-4403-B034-291A80FBDDB1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9c30d4e8-d9db-43d6-83e2-c08e4749ca29"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1f3c66e0-7684-4412-85ae-938bcfc42664"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0507654c-1543-47e1-81c5-300c2627be14}" enabled="1" method="Standard" siteId="{5a7cc8ab-a4dc-4f9b-bf60-66714049ad62}" removed="0"/>

</xml_diff>